<commit_message>
Actualizacao da pagina de boas praticas para presencas
</commit_message>
<xml_diff>
--- a/Selecionados_Motivacional_Ribaue_2026.xlsx
+++ b/Selecionados_Motivacional_Ribaue_2026.xlsx
@@ -102358,19 +102358,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="481cb719fb2f51215cc00c8d40533043">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="71df0815368817fe9627576b1e062219" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Criar um novo documento." ma:contentTypeScope="" ma:versionID="9a7078cd21229583650f2264465a1c40">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4e45437c47114f519c494620e3e4bb67" ns2:_="" ns3:_="">
     <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
     <xsd:import namespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
     <xsd:element name="properties">
@@ -102443,7 +102441,7 @@
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de Imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -102466,7 +102464,7 @@
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Partilhado Com" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -102485,7 +102483,7 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Detalhes de Partilhado Com" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
@@ -102513,8 +102511,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -102604,15 +102602,29 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7FAAC4-DCCC-45D2-BE24-F32F04F78BEF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{675D1D34-F605-4D6E-97B6-E03752A395F3}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3338ADEC-8CAE-41B2-8D8F-5460C83CEB8B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -102621,16 +102633,4 @@
     <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{212EFCB9-6160-46C4-9327-D087D97EA86F}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7FAAC4-DCCC-45D2-BE24-F32F04F78BEF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>